<commit_message>
Plots name a minor code updates
</commit_message>
<xml_diff>
--- a/Comparisons of RCA depth contours with NGDC bath/Box & Whisker plot for densified vertices.xlsx
+++ b/Comparisons of RCA depth contours with NGDC bath/Box & Whisker plot for densified vertices.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11010"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blake.feist/Documents/R/RCAs/Comparisons of NOAA depth contours with NGDC bath/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blake.feist/Documents/GitHub/RCA_closure_areas/Comparisons of RCA depth contours with NGDC bath/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D0E7B9-0786-7743-BCA0-C11B04251837}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88F77F5-4B0B-6740-BC40-5E19C7C354D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-50260" yWindow="460" windowWidth="50260" windowHeight="28340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-50120" yWindow="460" windowWidth="50120" windowHeight="28340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chart1" sheetId="2" r:id="rId1"/>
     <sheet name="Results" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="125725"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -97,7 +96,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.########"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -111,15 +110,23 @@
     </font>
     <font>
       <i/>
-      <sz val="10"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -160,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -171,22 +178,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -17518,30 +17531,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DN2586"/>
+  <dimension ref="A1:T2586"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="2" width="11.5" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="10" width="14" style="1" customWidth="1"/>
     <col min="11" max="20" width="11.5" style="1" customWidth="1"/>
     <col min="21" max="16384" width="11.5" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
       <c r="M1" s="1" t="s">
         <v>1</v>
       </c>
@@ -18098,34 +18111,34 @@
       </c>
     </row>
     <row r="28" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="H28" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="I28" s="4" t="s">
+      <c r="I28" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J28" s="4" t="s">
+      <c r="J28" s="5" t="s">
         <v>21</v>
       </c>
       <c r="Q28" s="2">
@@ -18142,34 +18155,34 @@
       </c>
     </row>
     <row r="29" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29" s="7">
         <v>616</v>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="8">
         <v>-59.457467532467497</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="8">
         <v>-204</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="8">
         <v>-121.8125</v>
       </c>
-      <c r="F29" s="6">
+      <c r="F29" s="8">
         <v>-71.356250000000003</v>
       </c>
-      <c r="G29" s="6">
+      <c r="G29" s="8">
         <v>-55.949999999999903</v>
       </c>
-      <c r="H29" s="6">
+      <c r="H29" s="8">
         <v>-40.387500000000003</v>
       </c>
-      <c r="I29" s="6">
+      <c r="I29" s="8">
         <v>-22.71875</v>
       </c>
-      <c r="J29" s="6">
+      <c r="J29" s="8">
         <v>-5.9</v>
       </c>
       <c r="O29" s="2">
@@ -18192,34 +18205,34 @@
       </c>
     </row>
     <row r="30" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30" s="7">
         <v>753</v>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="8">
         <v>-94.849667994687906</v>
       </c>
-      <c r="D30" s="6">
+      <c r="D30" s="8">
         <v>-368</v>
       </c>
-      <c r="E30" s="6">
+      <c r="E30" s="8">
         <v>-198.92500000000001</v>
       </c>
-      <c r="F30" s="6">
+      <c r="F30" s="8">
         <v>-114.3125</v>
       </c>
-      <c r="G30" s="6">
+      <c r="G30" s="8">
         <v>-80.800000000000097</v>
       </c>
-      <c r="H30" s="6">
+      <c r="H30" s="8">
         <v>-61.96875</v>
       </c>
-      <c r="I30" s="6">
+      <c r="I30" s="8">
         <v>-39.107500000000002</v>
       </c>
-      <c r="J30" s="6">
+      <c r="J30" s="8">
         <v>-11.4</v>
       </c>
       <c r="O30" s="2">
@@ -18236,34 +18249,34 @@
       </c>
     </row>
     <row r="31" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="7">
         <v>1111</v>
       </c>
-      <c r="C31" s="6">
+      <c r="C31" s="8">
         <v>-126.12880288028801</v>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="8">
         <v>-421</v>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="8">
         <v>-278.0625</v>
       </c>
-      <c r="F31" s="6">
+      <c r="F31" s="8">
         <v>-151.88749999999999</v>
       </c>
-      <c r="G31" s="6">
+      <c r="G31" s="8">
         <v>-110.1</v>
       </c>
-      <c r="H31" s="6">
+      <c r="H31" s="8">
         <v>-82.318749999999994</v>
       </c>
-      <c r="I31" s="6">
+      <c r="I31" s="8">
         <v>-50.487499999999997</v>
       </c>
-      <c r="J31" s="6">
+      <c r="J31" s="8">
         <v>0</v>
       </c>
       <c r="O31" s="2">
@@ -18286,34 +18299,34 @@
       </c>
     </row>
     <row r="32" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="5" t="s">
+      <c r="A32" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="7">
         <v>1236</v>
       </c>
-      <c r="C32" s="6">
+      <c r="C32" s="8">
         <v>-151.627184466019</v>
       </c>
-      <c r="D32" s="6">
+      <c r="D32" s="8">
         <v>-421</v>
       </c>
-      <c r="E32" s="6">
+      <c r="E32" s="8">
         <v>-312.72500000000002</v>
       </c>
-      <c r="F32" s="6">
+      <c r="F32" s="8">
         <v>-198.75624999999999</v>
       </c>
-      <c r="G32" s="6">
+      <c r="G32" s="8">
         <v>-125.65</v>
       </c>
-      <c r="H32" s="6">
+      <c r="H32" s="8">
         <v>-94.743750000000006</v>
       </c>
-      <c r="I32" s="6">
+      <c r="I32" s="8">
         <v>-59.737499999999997</v>
       </c>
-      <c r="J32" s="6">
+      <c r="J32" s="8">
         <v>-13.7</v>
       </c>
       <c r="O32" s="2">
@@ -18336,34 +18349,34 @@
       </c>
     </row>
     <row r="33" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B33" s="2">
+      <c r="B33" s="7">
         <v>1599</v>
       </c>
-      <c r="C33" s="6">
+      <c r="C33" s="8">
         <v>-178.96873045653501</v>
       </c>
-      <c r="D33" s="6">
+      <c r="D33" s="8">
         <v>-468</v>
       </c>
-      <c r="E33" s="6">
+      <c r="E33" s="8">
         <v>-347.66250000000002</v>
       </c>
-      <c r="F33" s="6">
+      <c r="F33" s="8">
         <v>-229.86250000000001</v>
       </c>
-      <c r="G33" s="6">
+      <c r="G33" s="8">
         <v>-158.1</v>
       </c>
-      <c r="H33" s="6">
+      <c r="H33" s="8">
         <v>-118.01875</v>
       </c>
-      <c r="I33" s="6">
+      <c r="I33" s="8">
         <v>-74.801249999999996</v>
       </c>
-      <c r="J33" s="6">
+      <c r="J33" s="8">
         <v>-54.5</v>
       </c>
       <c r="O33" s="2">
@@ -18380,34 +18393,34 @@
       </c>
     </row>
     <row r="34" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B34" s="2">
+      <c r="B34" s="7">
         <v>2274</v>
       </c>
-      <c r="C34" s="6">
+      <c r="C34" s="8">
         <v>-238.19582233949001</v>
       </c>
-      <c r="D34" s="6">
+      <c r="D34" s="8">
         <v>-607</v>
       </c>
-      <c r="E34" s="6">
+      <c r="E34" s="8">
         <v>-441.1825</v>
       </c>
-      <c r="F34" s="6">
+      <c r="F34" s="8">
         <v>-301.40625</v>
       </c>
-      <c r="G34" s="6">
+      <c r="G34" s="8">
         <v>-217.15</v>
       </c>
-      <c r="H34" s="6">
+      <c r="H34" s="8">
         <v>-160.19374999999999</v>
       </c>
-      <c r="I34" s="6">
+      <c r="I34" s="8">
         <v>-104.90875</v>
       </c>
-      <c r="J34" s="6">
+      <c r="J34" s="8">
         <v>-65.8</v>
       </c>
       <c r="O34" s="2">
@@ -18424,34 +18437,34 @@
       </c>
     </row>
     <row r="35" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35" s="7">
         <v>2859</v>
       </c>
-      <c r="C35" s="6">
+      <c r="C35" s="8">
         <v>-288.68842252535899</v>
       </c>
-      <c r="D35" s="6">
+      <c r="D35" s="8">
         <v>-690</v>
       </c>
-      <c r="E35" s="6">
+      <c r="E35" s="8">
         <v>-501.66250000000002</v>
       </c>
-      <c r="F35" s="6">
+      <c r="F35" s="8">
         <v>-361.16250000000002</v>
       </c>
-      <c r="G35" s="6">
+      <c r="G35" s="8">
         <v>-271.2</v>
       </c>
-      <c r="H35" s="6">
+      <c r="H35" s="8">
         <v>-199.61875000000001</v>
       </c>
-      <c r="I35" s="6">
+      <c r="I35" s="8">
         <v>-136.03375</v>
       </c>
-      <c r="J35" s="6">
+      <c r="J35" s="8">
         <v>-74</v>
       </c>
       <c r="O35" s="2">
@@ -18468,34 +18481,34 @@
       </c>
     </row>
     <row r="36" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B36" s="2">
+      <c r="B36" s="7">
         <v>3210</v>
       </c>
-      <c r="C36" s="6">
+      <c r="C36" s="8">
         <v>-333.44448598130799</v>
       </c>
-      <c r="D36" s="6">
+      <c r="D36" s="8">
         <v>-816</v>
       </c>
-      <c r="E36" s="6">
+      <c r="E36" s="8">
         <v>-556.09</v>
       </c>
-      <c r="F36" s="6">
+      <c r="F36" s="8">
         <v>-414.00625000000002</v>
       </c>
-      <c r="G36" s="6">
+      <c r="G36" s="8">
         <v>-316.75</v>
       </c>
-      <c r="H36" s="6">
+      <c r="H36" s="8">
         <v>-236.49375000000001</v>
       </c>
-      <c r="I36" s="6">
+      <c r="I36" s="8">
         <v>-158.97749999999999</v>
       </c>
-      <c r="J36" s="6">
+      <c r="J36" s="8">
         <v>-95</v>
       </c>
       <c r="O36" s="2">
@@ -18512,34 +18525,34 @@
       </c>
     </row>
     <row r="37" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B37" s="7">
         <v>3736</v>
       </c>
-      <c r="C37" s="6">
+      <c r="C37" s="8">
         <v>-393.14978586723799</v>
       </c>
-      <c r="D37" s="6">
+      <c r="D37" s="8">
         <v>-994.6</v>
       </c>
-      <c r="E37" s="6">
+      <c r="E37" s="8">
         <v>-681.16250000000002</v>
       </c>
-      <c r="F37" s="6">
+      <c r="F37" s="8">
         <v>-484.36874999999998</v>
       </c>
-      <c r="G37" s="6">
+      <c r="G37" s="8">
         <v>-369.05</v>
       </c>
-      <c r="H37" s="6">
+      <c r="H37" s="8">
         <v>-275.24374999999998</v>
       </c>
-      <c r="I37" s="6">
+      <c r="I37" s="8">
         <v>-190.13749999999999</v>
       </c>
-      <c r="J37" s="6">
+      <c r="J37" s="8">
         <v>-106</v>
       </c>
       <c r="O37" s="2">
@@ -18556,34 +18569,34 @@
       </c>
     </row>
     <row r="38" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B38" s="2">
+      <c r="B38" s="7">
         <v>3962</v>
       </c>
-      <c r="C38" s="6">
+      <c r="C38" s="8">
         <v>-454.07693084300899</v>
       </c>
-      <c r="D38" s="6">
+      <c r="D38" s="8">
         <v>-1217</v>
       </c>
-      <c r="E38" s="6">
+      <c r="E38" s="8">
         <v>-845.53750000000002</v>
       </c>
-      <c r="F38" s="6">
+      <c r="F38" s="8">
         <v>-553.30624999999998</v>
       </c>
-      <c r="G38" s="6">
+      <c r="G38" s="8">
         <v>-417.75</v>
       </c>
-      <c r="H38" s="6">
+      <c r="H38" s="8">
         <v>-317.49374999999998</v>
       </c>
-      <c r="I38" s="6">
+      <c r="I38" s="8">
         <v>-212.9975</v>
       </c>
-      <c r="J38" s="6">
+      <c r="J38" s="8">
         <v>-135</v>
       </c>
       <c r="O38" s="2">
@@ -18600,34 +18613,34 @@
       </c>
     </row>
     <row r="39" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A39" s="7" t="s">
+      <c r="A39" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B39" s="3">
+      <c r="B39" s="10">
         <v>4398</v>
       </c>
-      <c r="C39" s="8">
+      <c r="C39" s="11">
         <v>-539.50463847203298</v>
       </c>
-      <c r="D39" s="8">
+      <c r="D39" s="11">
         <v>-1218</v>
       </c>
-      <c r="E39" s="8">
+      <c r="E39" s="11">
         <v>-891.42750000000001</v>
       </c>
-      <c r="F39" s="8">
+      <c r="F39" s="11">
         <v>-645.50625000000002</v>
       </c>
-      <c r="G39" s="8">
+      <c r="G39" s="11">
         <v>-514.95000000000005</v>
       </c>
-      <c r="H39" s="8">
+      <c r="H39" s="11">
         <v>-404.29374999999999</v>
       </c>
-      <c r="I39" s="8">
+      <c r="I39" s="11">
         <v>-288.44375000000002</v>
       </c>
-      <c r="J39" s="8">
+      <c r="J39" s="11">
         <v>-137.6</v>
       </c>
       <c r="O39" s="2">

</xml_diff>